<commit_message>
Y9 Algebra strand complete: 07-18 published; log closeout
</commit_message>
<xml_diff>
--- a/lessonmap.xlsx
+++ b/lessonmap.xlsx
@@ -10849,12 +10849,22 @@
       </c>
       <c r="N129" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_07_gradient_of_a_line_segment_v2.html</t>
         </is>
       </c>
       <c r="Q129" s="15" t="inlineStr">
         <is>
-          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-03. Gradient given its own lesson under the 18-plan.</t>
+          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-03. Gradient given its own lesson under the 18-plan.</t>
         </is>
       </c>
     </row>
@@ -10922,12 +10932,22 @@
       </c>
       <c r="N130" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="Q130" t="inlineStr">
-        <is>
-          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-03. Builds on Y8 Pythagoras (y8_mea_11).</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_08_midpoint_and_distance_v2.html</t>
+        </is>
+      </c>
+      <c r="Q130" s="15" t="inlineStr">
+        <is>
+          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-03. Builds on Y8 Pythagoras (y8_mea_11).</t>
         </is>
       </c>
     </row>
@@ -10995,12 +11015,22 @@
       </c>
       <c r="N131" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_09_parallel_and_perpendicular_lines_v2.html</t>
         </is>
       </c>
       <c r="Q131" s="15" t="inlineStr">
         <is>
-          <t>NEW gap-fill: A03 elaboration 2 (parallel/perpendicular) was uncovered in the earlier 13-lesson build. Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-03.</t>
+          <t>NEW gap-fill: A03 elaboration 2 (parallel/perpendicular) was uncovered in the earlier 13-lesson build. Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-03.</t>
         </is>
       </c>
     </row>
@@ -11068,12 +11098,22 @@
       </c>
       <c r="N132" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_10_graphing_quadratic_functions_v2.html</t>
         </is>
       </c>
       <c r="Q132" s="15" t="inlineStr">
         <is>
-          <t>Watershed: first formal non-linear function. Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-03.</t>
+          <t>Watershed: first formal non-linear function. Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-03.</t>
         </is>
       </c>
     </row>
@@ -11141,12 +11181,22 @@
       </c>
       <c r="N133" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_11_solving_quadratics_graphically_v2.html</t>
         </is>
       </c>
       <c r="Q133" s="15" t="inlineStr">
         <is>
-          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Moon-phase elaboration 7 added. Batch y9-alg-04.</t>
+          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Moon-phase elaboration 7 added. Batch y9-alg-04.</t>
         </is>
       </c>
     </row>
@@ -11214,12 +11264,22 @@
       </c>
       <c r="N134" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_12_solving_monic_quadratics_algebraically_v2.html</t>
         </is>
       </c>
       <c r="Q134" s="15" t="inlineStr">
         <is>
-          <t>Parabola figure added (fix - was the one solving lesson with no figure). Null factor law folded in here. Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-04.</t>
+          <t>Parabola figure added (fix - was the one solving lesson with no figure). Null factor law folded in here. Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-04.</t>
         </is>
       </c>
     </row>
@@ -11287,12 +11347,22 @@
       </c>
       <c r="N135" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_13_modelling_with_linear_functions_v2.html</t>
         </is>
       </c>
       <c r="Q135" s="15" t="inlineStr">
         <is>
-          <t>A05 restored to 3 lessons under the 18-plan (was 1 combined lesson). Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-05.</t>
+          <t>A05 restored to 3 lessons under the 18-plan (was 1 combined lesson). Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-05.</t>
         </is>
       </c>
     </row>
@@ -11360,12 +11430,22 @@
       </c>
       <c r="N136" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_14_modelling_with_quadratic_functions_v2.html</t>
         </is>
       </c>
       <c r="Q136" s="15" t="inlineStr">
         <is>
-          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-05.</t>
+          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-05.</t>
         </is>
       </c>
     </row>
@@ -11433,12 +11513,22 @@
       </c>
       <c r="N137" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_15_choosing_linear_or_quadratic_models_v2.html</t>
         </is>
       </c>
       <c r="Q137" s="15" t="inlineStr">
         <is>
-          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-05.</t>
+          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-05.</t>
         </is>
       </c>
     </row>
@@ -11506,12 +11596,22 @@
       </c>
       <c r="N138" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_16_transformations_of_linear_graphs_v2.html</t>
         </is>
       </c>
       <c r="Q138" s="15" t="inlineStr">
         <is>
-          <t>A06 restored to 3 lessons under the 18-plan (was 1 combined lesson). Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-06.</t>
+          <t>A06 restored to 3 lessons under the 18-plan (was 1 combined lesson). Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-06.</t>
         </is>
       </c>
     </row>
@@ -11579,12 +11679,22 @@
       </c>
       <c r="N139" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_17_transformations_of_quadratic_graphs_v2.html</t>
         </is>
       </c>
       <c r="Q139" s="15" t="inlineStr">
         <is>
-          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-06.</t>
+          <t>Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-06.</t>
         </is>
       </c>
     </row>
@@ -11645,19 +11755,29 @@
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M140" t="inlineStr">
+      <c r="M140" s="15" t="inlineStr">
         <is>
           <t>y9_alg_16,y9_alg_17</t>
         </is>
       </c>
       <c r="N140" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/algebra/y9_alg_18_families_of_functions_v2.html</t>
         </is>
       </c>
       <c r="Q140" s="15" t="inlineStr">
         <is>
-          <t>NEW gap-fill: A06 elaboration 3 (function families) was uncovered in the earlier 13-lesson build. Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Status Planned; tags/elaborations to be confirmed from file &lt;meta&gt; at build closeout. Batch y9-alg-06.</t>
+          <t>NEW gap-fill: A06 elaboration 3 (function families) was uncovered in the earlier 13-lesson build. Re-mapped 2026-06-01 to the 18-lesson Y9 Algebra plan (go-18 decision). Built and published; metadata confirmed present in file &lt;meta&gt; per generation summary. Batch y9-alg-06.</t>
         </is>
       </c>
     </row>
@@ -11943,7 +12063,7 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="Q144" t="inlineStr">
+      <c r="Q144" s="15" t="inlineStr">
         <is>
           <t>Cross-strand prereq: needs y9_alg_01 negative exponents. Important sequencing — Algebra first, then Measurement.</t>
         </is>
@@ -12221,7 +12341,7 @@
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M148" t="inlineStr">
+      <c r="M148" s="15" t="inlineStr">
         <is>
           <t>y9_mea_06,y9_mea_07</t>
         </is>
@@ -12231,7 +12351,7 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="Q148" t="inlineStr">
+      <c r="Q148" s="15" t="inlineStr">
         <is>
           <t>Integration lesson — open-ended practice fits the conjecture/investigation flavour.</t>
         </is>
@@ -12358,7 +12478,7 @@
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M150" t="inlineStr">
+      <c r="M150" s="15" t="inlineStr">
         <is>
           <t>y9_mea_09</t>
         </is>
@@ -12433,7 +12553,7 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="Q151" t="inlineStr">
+      <c r="Q151" s="15" t="inlineStr">
         <is>
           <t>Extends Y8 mea_14 scale and proportion work; Y9 adds the formal modelling cycle.</t>
         </is>
@@ -12496,7 +12616,7 @@
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M152" t="inlineStr">
+      <c r="M152" s="15" t="inlineStr">
         <is>
           <t>y9_mea_11</t>
         </is>
@@ -12707,7 +12827,7 @@
           <t>auto-marked</t>
         </is>
       </c>
-      <c r="M155" t="inlineStr">
+      <c r="M155" s="15" t="inlineStr">
         <is>
           <t>y9_spa_02</t>
         </is>
@@ -12849,7 +12969,7 @@
           <t>auto-marked</t>
         </is>
       </c>
-      <c r="M157" t="inlineStr">
+      <c r="M157" s="15" t="inlineStr">
         <is>
           <t>y9_spa_04</t>
         </is>
@@ -12928,7 +13048,7 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="Q158" t="inlineStr">
+      <c r="Q158" s="15" t="inlineStr">
         <is>
           <t>Strategy-MCQ matches the decision-tree algorithm-design content.</t>
         </is>
@@ -12991,7 +13111,7 @@
           <t>strategy-MCQ</t>
         </is>
       </c>
-      <c r="M159" t="inlineStr">
+      <c r="M159" s="15" t="inlineStr">
         <is>
           <t>y9_spa_06</t>
         </is>
@@ -13129,7 +13249,7 @@
           <t>strategy-MCQ</t>
         </is>
       </c>
-      <c r="M161" t="inlineStr">
+      <c r="M161" s="15" t="inlineStr">
         <is>
           <t>y9_sta_01</t>
         </is>
@@ -13208,7 +13328,7 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="Q162" t="inlineStr">
+      <c r="Q162" s="15" t="inlineStr">
         <is>
           <t>Builds on Y8 sta_04/05 sampling and distribution work.</t>
         </is>
@@ -13413,7 +13533,7 @@
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M165" t="inlineStr">
+      <c r="M165" s="15" t="inlineStr">
         <is>
           <t>y9_sta_05</t>
         </is>
@@ -13565,7 +13685,7 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="Q167" t="inlineStr">
+      <c r="Q167" s="15" t="inlineStr">
         <is>
           <t>With/without replacement is the watershed concept — introduces conditional probability informally.</t>
         </is>
@@ -13697,7 +13817,7 @@
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M169" t="inlineStr">
+      <c r="M169" s="15" t="inlineStr">
         <is>
           <t>y9_pro_02,y9_pro_03</t>
         </is>
@@ -13839,7 +13959,7 @@
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M171" t="inlineStr">
+      <c r="M171" s="15" t="inlineStr">
         <is>
           <t>y10_num_01</t>
         </is>
@@ -14127,7 +14247,7 @@
           <t>auto-marked</t>
         </is>
       </c>
-      <c r="M175" t="inlineStr">
+      <c r="M175" s="15" t="inlineStr">
         <is>
           <t>y10_alg_02,y10_alg_03</t>
         </is>
@@ -14858,7 +14978,7 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="Q185" t="inlineStr">
+      <c r="Q185" s="15" t="inlineStr">
         <is>
           <t>Synthesis lesson — pulls together diagnostic skills from Y8 alg_05 (linear), Y9 alg_09 (quadratic) and y10_alg_11 (exponential).</t>
         </is>
@@ -16377,7 +16497,7 @@
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M206" t="inlineStr">
+      <c r="M206" s="15" t="inlineStr">
         <is>
           <t>y10_spa_02,y8_spa_03</t>
         </is>
@@ -17558,12 +17678,12 @@
       </c>
     </row>
     <row r="223" ht="15" customHeight="1" s="16">
-      <c r="A223" t="inlineStr">
+      <c r="A223" s="15" t="inlineStr">
         <is>
           <t>y10_pro_04</t>
         </is>
       </c>
-      <c r="B223" t="n">
+      <c r="B223" s="15" t="n">
         <v>10</v>
       </c>
       <c r="C223" s="15" t="inlineStr">
@@ -17571,25 +17691,25 @@
           <t>Probability</t>
         </is>
       </c>
-      <c r="D223" t="n">
+      <c r="D223" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E223" t="inlineStr">
+      <c r="E223" s="15" t="inlineStr">
         <is>
           <t>counter_intuitive_and_decision_simulations</t>
         </is>
       </c>
-      <c r="F223" t="inlineStr">
+      <c r="F223" s="15" t="inlineStr">
         <is>
           <t>y10_pro_04_counter_intuitive_and_decision_simulations_v2.html</t>
         </is>
       </c>
-      <c r="G223" t="inlineStr">
+      <c r="G223" s="15" t="inlineStr">
         <is>
           <t>AC9M10P02</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr">
+      <c r="H223" s="15" t="inlineStr">
         <is>
           <t>3,4,5</t>
         </is>
@@ -17599,32 +17719,32 @@
           <t>Strict</t>
         </is>
       </c>
-      <c r="J223" t="inlineStr">
+      <c r="J223" s="15" t="inlineStr">
         <is>
           <t>The likelihood of an event occurring can be affected by another event that has already taken place</t>
         </is>
       </c>
-      <c r="K223" t="inlineStr">
+      <c r="K223" s="15" t="inlineStr">
         <is>
           <t>Use simulations to gather data on counter-intuitive probability situations — the Monty Hall (three-door) problem and the birthday problem; identify situations in real life where probability simulations support decision-making such as queueing theory, insurance risk pricing and supply-and-demand for a product; use simulation to predict the number of people likely to be infected with a flu strain or virus.</t>
         </is>
       </c>
-      <c r="L223" t="inlineStr">
+      <c r="L223" s="15" t="inlineStr">
         <is>
           <t>auto-marked + open-ended</t>
         </is>
       </c>
-      <c r="M223" t="inlineStr">
+      <c r="M223" s="15" t="inlineStr">
         <is>
           <t>y10_pro_03</t>
         </is>
       </c>
-      <c r="N223" t="inlineStr">
+      <c r="N223" s="15" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="Q223" t="inlineStr">
+      <c r="Q223" s="15" t="inlineStr">
         <is>
           <t>Capstone probability lesson for Y10 — combines famous counter-intuitive problems with applied decision-making contexts. Builds on simulation work from Y7 pro_03, Y8 pro_04, Y9 pro_04.</t>
         </is>

</xml_diff>

<commit_message>
Mark y10_alg_01-10 Published (Batch 1 live)
</commit_message>
<xml_diff>
--- a/lessonmap.xlsx
+++ b/lessonmap.xlsx
@@ -10344,7 +10344,7 @@
           <t>auto-marked</t>
         </is>
       </c>
-      <c r="M123" t="inlineStr">
+      <c r="M123" s="15" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -10354,12 +10354,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O123" t="inlineStr">
+      <c r="O123" s="15" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="P123" t="inlineStr">
+      <c r="P123" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-9/algebra/y9_alg_01_index_laws_product_quotient_power_v2.html</t>
         </is>
@@ -10437,17 +10437,17 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O124" t="inlineStr">
+      <c r="O124" s="15" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="P124" t="inlineStr">
+      <c r="P124" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-9/algebra/y9_alg_02_zero_and_negative_indices_v2.html</t>
         </is>
       </c>
-      <c r="Q124" t="inlineStr">
+      <c r="Q124" s="15" t="inlineStr">
         <is>
           <t>Built 2026-05-31 (remote batch y9-alg-01). Covers planned-01 negative_integer_exponents content.</t>
         </is>
@@ -10510,7 +10510,7 @@
           <t>auto-marked</t>
         </is>
       </c>
-      <c r="M125" t="inlineStr">
+      <c r="M125" s="15" t="inlineStr">
         <is>
           <t>y9_alg_02</t>
         </is>
@@ -10520,12 +10520,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O125" t="inlineStr">
+      <c r="O125" s="15" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="P125" t="inlineStr">
+      <c r="P125" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-9/algebra/y9_alg_03_index_laws_with_variables_v2.html</t>
         </is>
@@ -10603,12 +10603,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O126" t="inlineStr">
+      <c r="O126" s="15" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="P126" t="inlineStr">
+      <c r="P126" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-9/algebra/y9_alg_04_expanding_binomial_products_v2.html</t>
         </is>
@@ -10686,12 +10686,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O127" t="inlineStr">
+      <c r="O127" s="15" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="P127" t="inlineStr">
+      <c r="P127" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-9/algebra/y9_alg_05_special_products_v2.html</t>
         </is>
@@ -10759,7 +10759,7 @@
           <t>auto-marked</t>
         </is>
       </c>
-      <c r="M128" t="inlineStr">
+      <c r="M128" s="15" t="inlineStr">
         <is>
           <t>y9_alg_05</t>
         </is>
@@ -10769,12 +10769,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O128" t="inlineStr">
+      <c r="O128" s="15" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="P128" t="inlineStr">
+      <c r="P128" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-9/algebra/y9_alg_06_factorising_monic_quadratics_v2.html</t>
         </is>
@@ -13820,7 +13820,17 @@
       </c>
       <c r="N171" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_01_expanding_special_products_and_non_monic_v2.html</t>
         </is>
       </c>
       <c r="Q171" s="15" t="inlineStr">
@@ -13893,7 +13903,17 @@
       </c>
       <c r="N172" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_02_factorising_quadratics_special_and_non_monic_v2.html</t>
         </is>
       </c>
       <c r="Q172" s="15" t="inlineStr">
@@ -13966,7 +13986,17 @@
       </c>
       <c r="N173" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_03_completing_the_square_v2.html</t>
         </is>
       </c>
       <c r="Q173" s="15" t="inlineStr">
@@ -14039,7 +14069,17 @@
       </c>
       <c r="N174" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_04_solving_quadratics_and_quadratic_formula_v2.html</t>
         </is>
       </c>
       <c r="Q174" s="15" t="inlineStr">
@@ -14107,7 +14147,17 @@
       </c>
       <c r="N175" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_05_simplifying_with_negative_exponents_and_variables_v2.html</t>
         </is>
       </c>
       <c r="Q175" s="15" t="inlineStr">
@@ -14175,7 +14225,17 @@
       </c>
       <c r="N176" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_06_solving_simultaneous_equations_graphically_v2.html</t>
         </is>
       </c>
       <c r="Q176" s="15" t="inlineStr">
@@ -14248,7 +14308,17 @@
       </c>
       <c r="N177" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_07_solving_simultaneous_equations_algebraically_v2.html</t>
         </is>
       </c>
       <c r="Q177" s="15" t="inlineStr">
@@ -14321,7 +14391,17 @@
       </c>
       <c r="N178" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_08_modelling_with_simultaneous_equations_v2.html</t>
         </is>
       </c>
       <c r="Q178" s="15" t="inlineStr">
@@ -14394,7 +14474,17 @@
       </c>
       <c r="N179" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_09_graphing_linear_inequalities_in_two_variables_v2.html</t>
         </is>
       </c>
       <c r="Q179" s="15" t="inlineStr">
@@ -14467,7 +14557,17 @@
       </c>
       <c r="N180" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_10_systems_of_inequalities_and_feasible_regions_v2.html</t>
         </is>
       </c>
       <c r="Q180" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Mark y10_alg_11-20 Published (Batch 2 live)
</commit_message>
<xml_diff>
--- a/lessonmap.xlsx
+++ b/lessonmap.xlsx
@@ -13823,12 +13823,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O171" t="inlineStr">
+      <c r="O171" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P171" t="inlineStr">
+      <c r="P171" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_01_expanding_special_products_and_non_monic_v2.html</t>
         </is>
@@ -13906,12 +13906,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O172" t="inlineStr">
+      <c r="O172" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P172" t="inlineStr">
+      <c r="P172" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_02_factorising_quadratics_special_and_non_monic_v2.html</t>
         </is>
@@ -13989,12 +13989,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O173" t="inlineStr">
+      <c r="O173" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P173" t="inlineStr">
+      <c r="P173" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_03_completing_the_square_v2.html</t>
         </is>
@@ -14072,12 +14072,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O174" t="inlineStr">
+      <c r="O174" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P174" t="inlineStr">
+      <c r="P174" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_04_solving_quadratics_and_quadratic_formula_v2.html</t>
         </is>
@@ -14150,12 +14150,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O175" t="inlineStr">
+      <c r="O175" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P175" t="inlineStr">
+      <c r="P175" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_05_simplifying_with_negative_exponents_and_variables_v2.html</t>
         </is>
@@ -14228,12 +14228,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O176" t="inlineStr">
+      <c r="O176" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P176" t="inlineStr">
+      <c r="P176" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_06_solving_simultaneous_equations_graphically_v2.html</t>
         </is>
@@ -14311,12 +14311,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O177" t="inlineStr">
+      <c r="O177" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P177" t="inlineStr">
+      <c r="P177" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_07_solving_simultaneous_equations_algebraically_v2.html</t>
         </is>
@@ -14394,12 +14394,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O178" t="inlineStr">
+      <c r="O178" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P178" t="inlineStr">
+      <c r="P178" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_08_modelling_with_simultaneous_equations_v2.html</t>
         </is>
@@ -14477,12 +14477,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O179" t="inlineStr">
+      <c r="O179" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P179" t="inlineStr">
+      <c r="P179" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_09_graphing_linear_inequalities_in_two_variables_v2.html</t>
         </is>
@@ -14560,12 +14560,12 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="O180" t="inlineStr">
+      <c r="O180" s="15" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="P180" t="inlineStr">
+      <c r="P180" s="15" t="inlineStr">
         <is>
           <t>https://seager94.github.io/year-10/algebra/y10_alg_10_systems_of_inequalities_and_feasible_regions_v2.html</t>
         </is>
@@ -14640,7 +14640,17 @@
       </c>
       <c r="N181" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_11_introducing_exponential_functions_v2.html</t>
         </is>
       </c>
       <c r="Q181" s="15" t="inlineStr">
@@ -14713,7 +14723,17 @@
       </c>
       <c r="N182" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_12_features_of_exponential_graphs_v2.html</t>
         </is>
       </c>
       <c r="Q182" s="15" t="inlineStr">
@@ -14786,7 +14806,17 @@
       </c>
       <c r="N183" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_13_solving_exponential_equations_v2.html</t>
         </is>
       </c>
       <c r="Q183" s="15" t="inlineStr">
@@ -14859,7 +14889,17 @@
       </c>
       <c r="N184" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_14_choosing_linear_quadratic_or_exponential_models_v2.html</t>
         </is>
       </c>
       <c r="Q184" s="15" t="inlineStr">
@@ -14932,7 +14972,17 @@
       </c>
       <c r="N185" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_15_exponential_growth_and_decay_v2.html</t>
         </is>
       </c>
     </row>
@@ -15000,7 +15050,17 @@
       </c>
       <c r="N186" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_16_compound_interest_modelling_v2.html</t>
         </is>
       </c>
       <c r="Q186" s="15" t="inlineStr">
@@ -15073,7 +15133,17 @@
       </c>
       <c r="N187" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_17_carbon_dating_and_applied_decay_modelling_v2.html</t>
         </is>
       </c>
       <c r="Q187" s="15" t="inlineStr">
@@ -15146,7 +15216,17 @@
       </c>
       <c r="N188" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_18_intersections_of_functions_with_digital_tools_v2.html</t>
         </is>
       </c>
       <c r="Q188" s="15" t="inlineStr">
@@ -15219,7 +15299,17 @@
       </c>
       <c r="N189" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_19_circle_equations_and_transformations_v2.html</t>
         </is>
       </c>
       <c r="Q189" s="15" t="inlineStr">
@@ -15292,7 +15382,17 @@
       </c>
       <c r="N190" s="15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-10/algebra/y10_alg_20_intervals_and_iterative_methods_v2.html</t>
         </is>
       </c>
       <c r="Q190" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Flip y8_sta_01-02 map rows to Published
</commit_message>
<xml_diff>
--- a/lessonmap.xlsx
+++ b/lessonmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sdavi\projects\seager94.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB84C048-9052-4CA4-9E74-A90C999118E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F4CA65C-DFA6-430A-9882-24FFD80CA077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4732" uniqueCount="1982">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4734" uniqueCount="1984">
   <si>
     <t>Lesson Map — AC9 Mathematics 7-10</t>
   </si>
@@ -5987,6 +5987,12 @@
   </si>
   <si>
     <t>y10_spa_02,y8_space_03</t>
+  </si>
+  <si>
+    <t>https://seager94.github.io/year-8/statistics/y8_sta_01_census_vs_sample_v2.html</t>
+  </si>
+  <si>
+    <t>https://seager94.github.io/year-8/statistics/y8_sta_02_identifying_and_avoiding_bias_v2.html</t>
   </si>
 </sst>
 </file>
@@ -6095,7 +6101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -6119,6 +6125,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12132,7 +12139,13 @@
         <v>403</v>
       </c>
       <c r="N111" s="1" t="s">
-        <v>411</v>
+        <v>66</v>
+      </c>
+      <c r="O111" s="13">
+        <v>46213</v>
+      </c>
+      <c r="P111" t="s">
+        <v>1982</v>
       </c>
       <c r="Q111" s="1" t="s">
         <v>767</v>
@@ -12179,7 +12192,13 @@
         <v>761</v>
       </c>
       <c r="N112" s="1" t="s">
-        <v>411</v>
+        <v>66</v>
+      </c>
+      <c r="O112" s="13">
+        <v>46213</v>
+      </c>
+      <c r="P112" t="s">
+        <v>1983</v>
       </c>
     </row>
     <row r="113" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -26410,7 +26429,7 @@
       </c>
       <c r="B5" s="1">
         <f>COUNTIF(Lessons!N2:N1000,"Planned")</f>
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -26446,7 +26465,7 @@
       </c>
       <c r="B9" s="1">
         <f>COUNTIF(Lessons!N2:N1000,"Published")</f>
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>